<commit_message>
School Management System Layout
</commit_message>
<xml_diff>
--- a/Presentation/New_Student_Management/Sources/Spreadsheets/candidate_list.xlsx
+++ b/Presentation/New_Student_Management/Sources/Spreadsheets/candidate_list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Projects\C# Projects\Student_Management\Sources\Spreadsheets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Projects\C# Projects\School_Management\Presentation\New_Student_Management\Sources\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{224361E3-168C-492D-962C-627A334DDD8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9676B3D2-2525-41B0-A6A0-706C83231FA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="4" xr2:uid="{E51BC222-ABB5-406A-BACB-6DFB53F1EC79}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="2" xr2:uid="{E51BC222-ABB5-406A-BACB-6DFB53F1EC79}"/>
   </bookViews>
   <sheets>
     <sheet name="Exam Room 1" sheetId="14" state="hidden" r:id="rId1"/>
@@ -55,6 +55,9 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -1149,7 +1152,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="119">
+  <cellXfs count="118">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1415,9 +1418,6 @@
     <xf numFmtId="165" fontId="27" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -1448,6 +1448,33 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="24" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1462,33 +1489,6 @@
     </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="3"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="24" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1827,99 +1827,99 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="96" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="97"/>
-      <c r="C1" s="97"/>
-      <c r="D1" s="97"/>
-      <c r="E1" s="97"/>
-      <c r="F1" s="97"/>
-      <c r="G1" s="97"/>
-      <c r="H1" s="97"/>
-      <c r="I1" s="97"/>
+      <c r="B1" s="96"/>
+      <c r="C1" s="96"/>
+      <c r="D1" s="96"/>
+      <c r="E1" s="96"/>
+      <c r="F1" s="96"/>
+      <c r="G1" s="96"/>
+      <c r="H1" s="96"/>
+      <c r="I1" s="96"/>
     </row>
     <row r="2" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="98" t="s">
+      <c r="A2" s="97" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="98"/>
-      <c r="C2" s="98"/>
-      <c r="D2" s="98"/>
-      <c r="E2" s="98"/>
-      <c r="F2" s="98"/>
-      <c r="G2" s="98"/>
-      <c r="H2" s="98"/>
-      <c r="I2" s="98"/>
+      <c r="B2" s="97"/>
+      <c r="C2" s="97"/>
+      <c r="D2" s="97"/>
+      <c r="E2" s="97"/>
+      <c r="F2" s="97"/>
+      <c r="G2" s="97"/>
+      <c r="H2" s="97"/>
+      <c r="I2" s="97"/>
     </row>
     <row r="3" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="99">
+      <c r="A3" s="98">
         <v>3</v>
       </c>
-      <c r="B3" s="99"/>
-      <c r="C3" s="99"/>
-      <c r="D3" s="99"/>
-      <c r="E3" s="99"/>
-      <c r="F3" s="99"/>
-      <c r="G3" s="99"/>
-      <c r="H3" s="99"/>
-      <c r="I3" s="99"/>
+      <c r="B3" s="98"/>
+      <c r="C3" s="98"/>
+      <c r="D3" s="98"/>
+      <c r="E3" s="98"/>
+      <c r="F3" s="98"/>
+      <c r="G3" s="98"/>
+      <c r="H3" s="98"/>
+      <c r="I3" s="98"/>
     </row>
     <row r="5" spans="1:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="94" t="s">
+      <c r="A5" s="93" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="94"/>
-      <c r="C5" s="94"/>
-      <c r="D5" s="94"/>
-      <c r="E5" s="94"/>
-      <c r="F5" s="94"/>
+      <c r="B5" s="93"/>
+      <c r="C5" s="93"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
     </row>
     <row r="6" spans="1:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="94" t="s">
+      <c r="A6" s="93" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="94"/>
-      <c r="C6" s="94"/>
-      <c r="D6" s="94"/>
-      <c r="E6" s="94"/>
-      <c r="F6" s="94"/>
+      <c r="B6" s="93"/>
+      <c r="C6" s="93"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
     </row>
     <row r="7" spans="1:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="94" t="s">
+      <c r="A7" s="93" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="94"/>
-      <c r="C7" s="94"/>
-      <c r="D7" s="94"/>
-      <c r="E7" s="94"/>
-      <c r="F7" s="94"/>
+      <c r="B7" s="93"/>
+      <c r="C7" s="93"/>
+      <c r="D7" s="93"/>
+      <c r="E7" s="93"/>
+      <c r="F7" s="93"/>
     </row>
     <row r="8" spans="1:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="95" t="s">
+      <c r="A8" s="94" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="95"/>
-      <c r="C8" s="95"/>
-      <c r="D8" s="95"/>
-      <c r="E8" s="95"/>
-      <c r="F8" s="95"/>
-      <c r="G8" s="95"/>
-      <c r="H8" s="95"/>
-      <c r="I8" s="95"/>
+      <c r="B8" s="94"/>
+      <c r="C8" s="94"/>
+      <c r="D8" s="94"/>
+      <c r="E8" s="94"/>
+      <c r="F8" s="94"/>
+      <c r="G8" s="94"/>
+      <c r="H8" s="94"/>
+      <c r="I8" s="94"/>
     </row>
     <row r="9" spans="1:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="96" t="s">
+      <c r="A9" s="95" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="96"/>
-      <c r="C9" s="96"/>
-      <c r="D9" s="96"/>
-      <c r="E9" s="96"/>
-      <c r="F9" s="96"/>
-      <c r="G9" s="96"/>
-      <c r="H9" s="96"/>
-      <c r="I9" s="96"/>
+      <c r="B9" s="95"/>
+      <c r="C9" s="95"/>
+      <c r="D9" s="95"/>
+      <c r="E9" s="95"/>
+      <c r="F9" s="95"/>
+      <c r="G9" s="95"/>
+      <c r="H9" s="95"/>
+      <c r="I9" s="95"/>
     </row>
     <row r="10" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="34" t="s">
@@ -2948,102 +2948,102 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="96" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="97"/>
-      <c r="C1" s="97"/>
-      <c r="D1" s="97"/>
-      <c r="E1" s="97"/>
-      <c r="F1" s="97"/>
-      <c r="G1" s="97"/>
-      <c r="H1" s="97"/>
-      <c r="I1" s="97"/>
+      <c r="B1" s="96"/>
+      <c r="C1" s="96"/>
+      <c r="D1" s="96"/>
+      <c r="E1" s="96"/>
+      <c r="F1" s="96"/>
+      <c r="G1" s="96"/>
+      <c r="H1" s="96"/>
+      <c r="I1" s="96"/>
     </row>
     <row r="2" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="98" t="s">
+      <c r="A2" s="97" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="98"/>
-      <c r="C2" s="98"/>
-      <c r="D2" s="98"/>
-      <c r="E2" s="98"/>
-      <c r="F2" s="98"/>
-      <c r="G2" s="98"/>
-      <c r="H2" s="98"/>
-      <c r="I2" s="98"/>
+      <c r="B2" s="97"/>
+      <c r="C2" s="97"/>
+      <c r="D2" s="97"/>
+      <c r="E2" s="97"/>
+      <c r="F2" s="97"/>
+      <c r="G2" s="97"/>
+      <c r="H2" s="97"/>
+      <c r="I2" s="97"/>
     </row>
     <row r="3" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="99">
+      <c r="A3" s="98">
         <v>3</v>
       </c>
-      <c r="B3" s="99"/>
-      <c r="C3" s="99"/>
-      <c r="D3" s="99"/>
-      <c r="E3" s="99"/>
-      <c r="F3" s="99"/>
-      <c r="G3" s="99"/>
-      <c r="H3" s="99"/>
-      <c r="I3" s="99"/>
+      <c r="B3" s="98"/>
+      <c r="C3" s="98"/>
+      <c r="D3" s="98"/>
+      <c r="E3" s="98"/>
+      <c r="F3" s="98"/>
+      <c r="G3" s="98"/>
+      <c r="H3" s="98"/>
+      <c r="I3" s="98"/>
     </row>
     <row r="4" spans="1:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A4" s="103" t="s">
+      <c r="A4" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="103"/>
-      <c r="C4" s="103"/>
-      <c r="D4" s="103"/>
-      <c r="E4" s="103"/>
-      <c r="F4" s="103"/>
+      <c r="B4" s="102"/>
+      <c r="C4" s="102"/>
+      <c r="D4" s="102"/>
+      <c r="E4" s="102"/>
+      <c r="F4" s="102"/>
       <c r="G4" s="31"/>
     </row>
     <row r="5" spans="1:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A5" s="103" t="s">
+      <c r="A5" s="102" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="103"/>
-      <c r="C5" s="103"/>
-      <c r="D5" s="103"/>
-      <c r="E5" s="103"/>
-      <c r="F5" s="103"/>
+      <c r="B5" s="102"/>
+      <c r="C5" s="102"/>
+      <c r="D5" s="102"/>
+      <c r="E5" s="102"/>
+      <c r="F5" s="102"/>
       <c r="G5" s="31"/>
     </row>
     <row r="6" spans="1:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="100" t="s">
+      <c r="A6" s="99" t="s">
         <v>104</v>
       </c>
-      <c r="B6" s="100"/>
-      <c r="C6" s="100"/>
-      <c r="D6" s="100"/>
-      <c r="E6" s="100"/>
-      <c r="F6" s="100"/>
+      <c r="B6" s="99"/>
+      <c r="C6" s="99"/>
+      <c r="D6" s="99"/>
+      <c r="E6" s="99"/>
+      <c r="F6" s="99"/>
       <c r="G6" s="30"/>
     </row>
     <row r="7" spans="1:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A7" s="101" t="s">
+      <c r="A7" s="100" t="s">
         <v>105</v>
       </c>
-      <c r="B7" s="101"/>
-      <c r="C7" s="101"/>
-      <c r="D7" s="101"/>
-      <c r="E7" s="101"/>
-      <c r="F7" s="101"/>
-      <c r="G7" s="101"/>
-      <c r="H7" s="101"/>
-      <c r="I7" s="101"/>
+      <c r="B7" s="100"/>
+      <c r="C7" s="100"/>
+      <c r="D7" s="100"/>
+      <c r="E7" s="100"/>
+      <c r="F7" s="100"/>
+      <c r="G7" s="100"/>
+      <c r="H7" s="100"/>
+      <c r="I7" s="100"/>
     </row>
     <row r="8" spans="1:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A8" s="102" t="s">
+      <c r="A8" s="101" t="s">
         <v>106</v>
       </c>
-      <c r="B8" s="102"/>
-      <c r="C8" s="102"/>
-      <c r="D8" s="102"/>
-      <c r="E8" s="102"/>
-      <c r="F8" s="102"/>
-      <c r="G8" s="102"/>
-      <c r="H8" s="102"/>
-      <c r="I8" s="102"/>
+      <c r="B8" s="101"/>
+      <c r="C8" s="101"/>
+      <c r="D8" s="101"/>
+      <c r="E8" s="101"/>
+      <c r="F8" s="101"/>
+      <c r="G8" s="101"/>
+      <c r="H8" s="101"/>
+      <c r="I8" s="101"/>
     </row>
     <row r="9" spans="1:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="34" t="s">
@@ -4015,156 +4015,156 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="113" t="s">
+      <c r="A1" s="103" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="113"/>
-      <c r="C1" s="113"/>
-      <c r="D1" s="113"/>
-      <c r="E1" s="113"/>
-      <c r="F1" s="113"/>
-      <c r="G1" s="113"/>
-      <c r="H1" s="113"/>
-      <c r="I1" s="113"/>
-      <c r="J1" s="113"/>
-      <c r="K1" s="113"/>
-      <c r="L1" s="113"/>
+      <c r="B1" s="103"/>
+      <c r="C1" s="103"/>
+      <c r="D1" s="103"/>
+      <c r="E1" s="103"/>
+      <c r="F1" s="103"/>
+      <c r="G1" s="103"/>
+      <c r="H1" s="103"/>
+      <c r="I1" s="103"/>
+      <c r="J1" s="103"/>
+      <c r="K1" s="103"/>
+      <c r="L1" s="103"/>
     </row>
     <row r="2" spans="1:12" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="114" t="s">
+      <c r="A2" s="104" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="115"/>
-      <c r="C2" s="115"/>
-      <c r="D2" s="115"/>
-      <c r="E2" s="115"/>
-      <c r="F2" s="115"/>
-      <c r="G2" s="115"/>
-      <c r="H2" s="115"/>
-      <c r="I2" s="115"/>
-      <c r="J2" s="115"/>
-      <c r="K2" s="115"/>
-      <c r="L2" s="115"/>
+      <c r="B2" s="105"/>
+      <c r="C2" s="105"/>
+      <c r="D2" s="105"/>
+      <c r="E2" s="105"/>
+      <c r="F2" s="105"/>
+      <c r="G2" s="105"/>
+      <c r="H2" s="105"/>
+      <c r="I2" s="105"/>
+      <c r="J2" s="105"/>
+      <c r="K2" s="105"/>
+      <c r="L2" s="105"/>
     </row>
     <row r="3" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="116">
+      <c r="A3" s="106">
         <v>3</v>
       </c>
-      <c r="B3" s="116"/>
-      <c r="C3" s="116"/>
-      <c r="D3" s="116"/>
-      <c r="E3" s="116"/>
-      <c r="F3" s="116"/>
-      <c r="G3" s="116"/>
-      <c r="H3" s="116"/>
-      <c r="I3" s="116"/>
-      <c r="J3" s="116"/>
-      <c r="K3" s="116"/>
-      <c r="L3" s="116"/>
+      <c r="B3" s="106"/>
+      <c r="C3" s="106"/>
+      <c r="D3" s="106"/>
+      <c r="E3" s="106"/>
+      <c r="F3" s="106"/>
+      <c r="G3" s="106"/>
+      <c r="H3" s="106"/>
+      <c r="I3" s="106"/>
+      <c r="J3" s="106"/>
+      <c r="K3" s="106"/>
+      <c r="L3" s="106"/>
     </row>
     <row r="4" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="117" t="s">
+      <c r="A4" s="107" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="117"/>
-      <c r="C4" s="117"/>
-      <c r="D4" s="117"/>
-      <c r="E4" s="117"/>
-      <c r="F4" s="117"/>
-      <c r="G4" s="117"/>
-      <c r="H4" s="117"/>
-      <c r="I4" s="117"/>
-      <c r="J4" s="117"/>
-      <c r="K4" s="117"/>
+      <c r="B4" s="107"/>
+      <c r="C4" s="107"/>
+      <c r="D4" s="107"/>
+      <c r="E4" s="107"/>
+      <c r="F4" s="107"/>
+      <c r="G4" s="107"/>
+      <c r="H4" s="107"/>
+      <c r="I4" s="107"/>
+      <c r="J4" s="107"/>
+      <c r="K4" s="107"/>
       <c r="L4" s="6"/>
     </row>
     <row r="5" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="117" t="s">
+      <c r="A5" s="107" t="s">
         <v>41</v>
       </c>
-      <c r="B5" s="117"/>
-      <c r="C5" s="117"/>
-      <c r="D5" s="117"/>
-      <c r="E5" s="117"/>
-      <c r="F5" s="117"/>
-      <c r="G5" s="117"/>
-      <c r="H5" s="117"/>
-      <c r="I5" s="117"/>
-      <c r="J5" s="117"/>
-      <c r="K5" s="117"/>
+      <c r="B5" s="107"/>
+      <c r="C5" s="107"/>
+      <c r="D5" s="107"/>
+      <c r="E5" s="107"/>
+      <c r="F5" s="107"/>
+      <c r="G5" s="107"/>
+      <c r="H5" s="107"/>
+      <c r="I5" s="107"/>
+      <c r="J5" s="107"/>
+      <c r="K5" s="107"/>
       <c r="L5" s="6"/>
     </row>
     <row r="6" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="109" t="s">
+      <c r="A6" s="108" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="109"/>
-      <c r="C6" s="109"/>
-      <c r="D6" s="109"/>
-      <c r="E6" s="109"/>
-      <c r="F6" s="109"/>
-      <c r="G6" s="109"/>
-      <c r="H6" s="109"/>
-      <c r="I6" s="109"/>
-      <c r="J6" s="109"/>
-      <c r="K6" s="109"/>
-      <c r="L6" s="109"/>
+      <c r="B6" s="108"/>
+      <c r="C6" s="108"/>
+      <c r="D6" s="108"/>
+      <c r="E6" s="108"/>
+      <c r="F6" s="108"/>
+      <c r="G6" s="108"/>
+      <c r="H6" s="108"/>
+      <c r="I6" s="108"/>
+      <c r="J6" s="108"/>
+      <c r="K6" s="108"/>
+      <c r="L6" s="108"/>
     </row>
     <row r="7" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="109" t="s">
+      <c r="A7" s="108" t="s">
         <v>176</v>
       </c>
-      <c r="B7" s="109"/>
-      <c r="C7" s="109"/>
-      <c r="D7" s="109"/>
-      <c r="E7" s="109"/>
-      <c r="F7" s="109"/>
-      <c r="G7" s="109"/>
-      <c r="H7" s="109"/>
-      <c r="I7" s="109"/>
-      <c r="J7" s="109"/>
-      <c r="K7" s="109"/>
-      <c r="L7" s="109"/>
+      <c r="B7" s="108"/>
+      <c r="C7" s="108"/>
+      <c r="D7" s="108"/>
+      <c r="E7" s="108"/>
+      <c r="F7" s="108"/>
+      <c r="G7" s="108"/>
+      <c r="H7" s="108"/>
+      <c r="I7" s="108"/>
+      <c r="J7" s="108"/>
+      <c r="K7" s="108"/>
+      <c r="L7" s="108"/>
     </row>
     <row r="8" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="110" t="s">
+      <c r="A8" s="109" t="s">
         <v>177</v>
       </c>
-      <c r="B8" s="110" t="s">
+      <c r="B8" s="109" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="110" t="s">
+      <c r="C8" s="109" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="110" t="s">
+      <c r="D8" s="109" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="111" t="s">
+      <c r="E8" s="110" t="s">
         <v>11</v>
       </c>
-      <c r="F8" s="110" t="s">
+      <c r="F8" s="109" t="s">
         <v>178</v>
       </c>
-      <c r="G8" s="112" t="s">
+      <c r="G8" s="111" t="s">
         <v>179</v>
       </c>
-      <c r="H8" s="110"/>
-      <c r="I8" s="110"/>
-      <c r="J8" s="110"/>
-      <c r="K8" s="110" t="s">
+      <c r="H8" s="109"/>
+      <c r="I8" s="109"/>
+      <c r="J8" s="109"/>
+      <c r="K8" s="109" t="s">
         <v>12</v>
       </c>
-      <c r="L8" s="110" t="s">
+      <c r="L8" s="109" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="25.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="110"/>
-      <c r="B9" s="110"/>
-      <c r="C9" s="110"/>
-      <c r="D9" s="110"/>
-      <c r="E9" s="111"/>
-      <c r="F9" s="110"/>
+      <c r="A9" s="109"/>
+      <c r="B9" s="109"/>
+      <c r="C9" s="109"/>
+      <c r="D9" s="109"/>
+      <c r="E9" s="110"/>
+      <c r="F9" s="109"/>
       <c r="G9" s="64" t="s">
         <v>180</v>
       </c>
@@ -4177,8 +4177,8 @@
       <c r="J9" s="61" t="s">
         <v>182</v>
       </c>
-      <c r="K9" s="110"/>
-      <c r="L9" s="110"/>
+      <c r="K9" s="109"/>
+      <c r="L9" s="109"/>
     </row>
     <row r="10" spans="1:12" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="62">
@@ -4198,7 +4198,7 @@
       </c>
       <c r="F10" s="67">
         <f ca="1">IF(E10 &lt;&gt; "",YEAR(NOW())-YEAR(E10), "")</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G10" s="90" t="s">
         <v>185</v>
@@ -4211,84 +4211,84 @@
       <c r="K10" s="63" t="s">
         <v>186</v>
       </c>
-      <c r="L10" s="93"/>
+      <c r="L10" s="63"/>
     </row>
     <row r="11" spans="1:12" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="106"/>
-      <c r="B11" s="106"/>
-      <c r="C11" s="106"/>
-      <c r="D11" s="106"/>
-      <c r="E11" s="106"/>
-      <c r="F11" s="106"/>
-      <c r="G11" s="106"/>
-      <c r="H11" s="106"/>
-      <c r="I11" s="106"/>
-      <c r="J11" s="106"/>
-      <c r="K11" s="106"/>
-      <c r="L11" s="106"/>
+      <c r="A11" s="114"/>
+      <c r="B11" s="114"/>
+      <c r="C11" s="114"/>
+      <c r="D11" s="114"/>
+      <c r="E11" s="114"/>
+      <c r="F11" s="114"/>
+      <c r="G11" s="114"/>
+      <c r="H11" s="114"/>
+      <c r="I11" s="114"/>
+      <c r="J11" s="114"/>
+      <c r="K11" s="114"/>
+      <c r="L11" s="114"/>
     </row>
     <row r="12" spans="1:12" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="28"/>
-      <c r="B12" s="107">
+      <c r="B12" s="115">
         <v>0</v>
       </c>
-      <c r="C12" s="107"/>
+      <c r="C12" s="115"/>
       <c r="D12" s="57"/>
       <c r="E12" s="65"/>
       <c r="F12" s="89"/>
-      <c r="G12" s="108" t="s">
+      <c r="G12" s="116" t="s">
         <v>187</v>
       </c>
-      <c r="H12" s="108"/>
-      <c r="I12" s="108"/>
-      <c r="J12" s="108"/>
-      <c r="K12" s="108"/>
-      <c r="L12" s="108"/>
+      <c r="H12" s="116"/>
+      <c r="I12" s="116"/>
+      <c r="J12" s="116"/>
+      <c r="K12" s="116"/>
+      <c r="L12" s="116"/>
     </row>
     <row r="13" spans="1:12" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="26"/>
-      <c r="B13" s="107">
+      <c r="B13" s="115">
         <v>0</v>
       </c>
-      <c r="C13" s="107"/>
-      <c r="G13" s="108" t="str">
+      <c r="C13" s="115"/>
+      <c r="G13" s="116" t="str">
         <f>_xlfn.CONCAT("   ដុនបូស្កូប៉ោយប៉ែត ថ្ងៃទី","១៣","   ខែ","កញ្ញា","    ឆ្នាំ","២០២៤")</f>
         <v xml:space="preserve">   ដុនបូស្កូប៉ោយប៉ែត ថ្ងៃទី១៣   ខែកញ្ញា    ឆ្នាំ២០២៤</v>
       </c>
-      <c r="H13" s="108"/>
-      <c r="I13" s="108"/>
-      <c r="J13" s="108"/>
-      <c r="K13" s="108"/>
-      <c r="L13" s="108"/>
+      <c r="H13" s="116"/>
+      <c r="I13" s="116"/>
+      <c r="J13" s="116"/>
+      <c r="K13" s="116"/>
+      <c r="L13" s="116"/>
     </row>
     <row r="14" spans="1:12" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="8"/>
       <c r="G14" s="74"/>
-      <c r="H14" s="104" t="s">
+      <c r="H14" s="112" t="s">
         <v>189</v>
       </c>
-      <c r="I14" s="104"/>
-      <c r="J14" s="104"/>
-      <c r="K14" s="104"/>
-      <c r="L14" s="104"/>
+      <c r="I14" s="112"/>
+      <c r="J14" s="112"/>
+      <c r="K14" s="112"/>
+      <c r="L14" s="112"/>
     </row>
     <row r="15" spans="1:12" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="28"/>
-      <c r="B15" s="105" t="s">
+      <c r="B15" s="113" t="s">
         <v>190</v>
       </c>
-      <c r="C15" s="105"/>
-      <c r="D15" s="105"/>
-      <c r="E15" s="105"/>
+      <c r="C15" s="113"/>
+      <c r="D15" s="113"/>
+      <c r="E15" s="113"/>
     </row>
     <row r="16" spans="1:12" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="28"/>
-      <c r="B16" s="104" t="s">
+      <c r="B16" s="112" t="s">
         <v>191</v>
       </c>
-      <c r="C16" s="104"/>
-      <c r="D16" s="104"/>
-      <c r="E16" s="104"/>
+      <c r="C16" s="112"/>
+      <c r="D16" s="112"/>
+      <c r="E16" s="112"/>
       <c r="F16" s="59"/>
       <c r="G16" s="59"/>
       <c r="H16" s="59"/>
@@ -4528,11 +4528,14 @@
     <sortCondition ref="B10"/>
   </sortState>
   <mergeCells count="24">
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
+    <mergeCell ref="H14:L14"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="B16:E16"/>
+    <mergeCell ref="A11:L11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="G12:L12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="G13:L13"/>
     <mergeCell ref="A6:L6"/>
     <mergeCell ref="A7:L7"/>
     <mergeCell ref="A8:A9"/>
@@ -4544,14 +4547,11 @@
     <mergeCell ref="G8:J8"/>
     <mergeCell ref="K8:K9"/>
     <mergeCell ref="L8:L9"/>
-    <mergeCell ref="H14:L14"/>
-    <mergeCell ref="B15:E15"/>
-    <mergeCell ref="B16:E16"/>
-    <mergeCell ref="A11:L11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="G12:L12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="G13:L13"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
@@ -4583,156 +4583,156 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="113" t="s">
+      <c r="A1" s="103" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="113"/>
-      <c r="C1" s="113"/>
-      <c r="D1" s="113"/>
-      <c r="E1" s="113"/>
-      <c r="F1" s="113"/>
-      <c r="G1" s="113"/>
-      <c r="H1" s="113"/>
-      <c r="I1" s="113"/>
-      <c r="J1" s="113"/>
-      <c r="K1" s="113"/>
-      <c r="L1" s="113"/>
+      <c r="B1" s="103"/>
+      <c r="C1" s="103"/>
+      <c r="D1" s="103"/>
+      <c r="E1" s="103"/>
+      <c r="F1" s="103"/>
+      <c r="G1" s="103"/>
+      <c r="H1" s="103"/>
+      <c r="I1" s="103"/>
+      <c r="J1" s="103"/>
+      <c r="K1" s="103"/>
+      <c r="L1" s="103"/>
     </row>
     <row r="2" spans="1:12" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="114" t="s">
+      <c r="A2" s="104" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="115"/>
-      <c r="C2" s="115"/>
-      <c r="D2" s="115"/>
-      <c r="E2" s="115"/>
-      <c r="F2" s="115"/>
-      <c r="G2" s="115"/>
-      <c r="H2" s="115"/>
-      <c r="I2" s="115"/>
-      <c r="J2" s="115"/>
-      <c r="K2" s="115"/>
-      <c r="L2" s="115"/>
+      <c r="B2" s="105"/>
+      <c r="C2" s="105"/>
+      <c r="D2" s="105"/>
+      <c r="E2" s="105"/>
+      <c r="F2" s="105"/>
+      <c r="G2" s="105"/>
+      <c r="H2" s="105"/>
+      <c r="I2" s="105"/>
+      <c r="J2" s="105"/>
+      <c r="K2" s="105"/>
+      <c r="L2" s="105"/>
     </row>
     <row r="3" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="116">
+      <c r="A3" s="106">
         <v>3</v>
       </c>
-      <c r="B3" s="116"/>
-      <c r="C3" s="116"/>
-      <c r="D3" s="116"/>
-      <c r="E3" s="116"/>
-      <c r="F3" s="116"/>
-      <c r="G3" s="116"/>
-      <c r="H3" s="116"/>
-      <c r="I3" s="116"/>
-      <c r="J3" s="116"/>
-      <c r="K3" s="116"/>
-      <c r="L3" s="116"/>
+      <c r="B3" s="106"/>
+      <c r="C3" s="106"/>
+      <c r="D3" s="106"/>
+      <c r="E3" s="106"/>
+      <c r="F3" s="106"/>
+      <c r="G3" s="106"/>
+      <c r="H3" s="106"/>
+      <c r="I3" s="106"/>
+      <c r="J3" s="106"/>
+      <c r="K3" s="106"/>
+      <c r="L3" s="106"/>
     </row>
     <row r="4" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="117" t="s">
+      <c r="A4" s="107" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="117"/>
-      <c r="C4" s="117"/>
-      <c r="D4" s="117"/>
-      <c r="E4" s="117"/>
-      <c r="F4" s="117"/>
-      <c r="G4" s="117"/>
-      <c r="H4" s="117"/>
-      <c r="I4" s="117"/>
-      <c r="J4" s="117"/>
-      <c r="K4" s="117"/>
+      <c r="B4" s="107"/>
+      <c r="C4" s="107"/>
+      <c r="D4" s="107"/>
+      <c r="E4" s="107"/>
+      <c r="F4" s="107"/>
+      <c r="G4" s="107"/>
+      <c r="H4" s="107"/>
+      <c r="I4" s="107"/>
+      <c r="J4" s="107"/>
+      <c r="K4" s="107"/>
       <c r="L4" s="6"/>
     </row>
     <row r="5" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="117" t="s">
+      <c r="A5" s="107" t="s">
         <v>41</v>
       </c>
-      <c r="B5" s="117"/>
-      <c r="C5" s="117"/>
-      <c r="D5" s="117"/>
-      <c r="E5" s="117"/>
-      <c r="F5" s="117"/>
-      <c r="G5" s="117"/>
-      <c r="H5" s="117"/>
-      <c r="I5" s="117"/>
-      <c r="J5" s="117"/>
-      <c r="K5" s="117"/>
+      <c r="B5" s="107"/>
+      <c r="C5" s="107"/>
+      <c r="D5" s="107"/>
+      <c r="E5" s="107"/>
+      <c r="F5" s="107"/>
+      <c r="G5" s="107"/>
+      <c r="H5" s="107"/>
+      <c r="I5" s="107"/>
+      <c r="J5" s="107"/>
+      <c r="K5" s="107"/>
       <c r="L5" s="6"/>
     </row>
     <row r="6" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="109" t="s">
+      <c r="A6" s="108" t="s">
         <v>192</v>
       </c>
-      <c r="B6" s="109"/>
-      <c r="C6" s="109"/>
-      <c r="D6" s="109"/>
-      <c r="E6" s="109"/>
-      <c r="F6" s="109"/>
-      <c r="G6" s="109"/>
-      <c r="H6" s="109"/>
-      <c r="I6" s="109"/>
-      <c r="J6" s="109"/>
-      <c r="K6" s="109"/>
-      <c r="L6" s="109"/>
+      <c r="B6" s="108"/>
+      <c r="C6" s="108"/>
+      <c r="D6" s="108"/>
+      <c r="E6" s="108"/>
+      <c r="F6" s="108"/>
+      <c r="G6" s="108"/>
+      <c r="H6" s="108"/>
+      <c r="I6" s="108"/>
+      <c r="J6" s="108"/>
+      <c r="K6" s="108"/>
+      <c r="L6" s="108"/>
     </row>
     <row r="7" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="109" t="s">
+      <c r="A7" s="108" t="s">
         <v>176</v>
       </c>
-      <c r="B7" s="109"/>
-      <c r="C7" s="109"/>
-      <c r="D7" s="109"/>
-      <c r="E7" s="109"/>
-      <c r="F7" s="109"/>
-      <c r="G7" s="109"/>
-      <c r="H7" s="109"/>
-      <c r="I7" s="109"/>
-      <c r="J7" s="109"/>
-      <c r="K7" s="109"/>
-      <c r="L7" s="109"/>
+      <c r="B7" s="108"/>
+      <c r="C7" s="108"/>
+      <c r="D7" s="108"/>
+      <c r="E7" s="108"/>
+      <c r="F7" s="108"/>
+      <c r="G7" s="108"/>
+      <c r="H7" s="108"/>
+      <c r="I7" s="108"/>
+      <c r="J7" s="108"/>
+      <c r="K7" s="108"/>
+      <c r="L7" s="108"/>
     </row>
     <row r="8" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="110" t="s">
+      <c r="A8" s="109" t="s">
         <v>177</v>
       </c>
-      <c r="B8" s="110" t="s">
+      <c r="B8" s="109" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="110" t="s">
+      <c r="C8" s="109" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="110" t="s">
+      <c r="D8" s="109" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="111" t="s">
+      <c r="E8" s="110" t="s">
         <v>11</v>
       </c>
-      <c r="F8" s="110" t="s">
+      <c r="F8" s="109" t="s">
         <v>178</v>
       </c>
-      <c r="G8" s="112" t="s">
+      <c r="G8" s="111" t="s">
         <v>179</v>
       </c>
-      <c r="H8" s="110"/>
-      <c r="I8" s="110"/>
-      <c r="J8" s="110"/>
-      <c r="K8" s="110" t="s">
+      <c r="H8" s="109"/>
+      <c r="I8" s="109"/>
+      <c r="J8" s="109"/>
+      <c r="K8" s="109" t="s">
         <v>12</v>
       </c>
-      <c r="L8" s="110" t="s">
+      <c r="L8" s="109" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="110"/>
-      <c r="B9" s="110"/>
-      <c r="C9" s="110"/>
-      <c r="D9" s="110"/>
-      <c r="E9" s="111"/>
-      <c r="F9" s="110"/>
+      <c r="A9" s="109"/>
+      <c r="B9" s="109"/>
+      <c r="C9" s="109"/>
+      <c r="D9" s="109"/>
+      <c r="E9" s="110"/>
+      <c r="F9" s="109"/>
       <c r="G9" s="70" t="s">
         <v>180</v>
       </c>
@@ -4745,10 +4745,10 @@
       <c r="J9" s="71" t="s">
         <v>182</v>
       </c>
-      <c r="K9" s="110"/>
-      <c r="L9" s="110"/>
-    </row>
-    <row r="10" spans="1:12" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K9" s="109"/>
+      <c r="L9" s="109"/>
+    </row>
+    <row r="10" spans="1:12" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="62">
         <v>1</v>
       </c>
@@ -4766,7 +4766,7 @@
       </c>
       <c r="F10" s="67">
         <f ca="1">IF(E10 &lt;&gt; "",YEAR(NOW())-YEAR(E10), "")</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G10" s="90" t="s">
         <v>185</v>
@@ -4779,83 +4779,83 @@
       <c r="K10" s="63" t="s">
         <v>186</v>
       </c>
-      <c r="L10" s="93"/>
+      <c r="L10" s="63"/>
     </row>
     <row r="11" spans="1:12" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="106"/>
-      <c r="B11" s="106"/>
-      <c r="C11" s="106"/>
-      <c r="D11" s="106"/>
-      <c r="E11" s="106"/>
-      <c r="F11" s="106"/>
-      <c r="G11" s="106"/>
-      <c r="H11" s="106"/>
-      <c r="I11" s="106"/>
-      <c r="J11" s="106"/>
-      <c r="K11" s="106"/>
-      <c r="L11" s="106"/>
+      <c r="A11" s="114"/>
+      <c r="B11" s="114"/>
+      <c r="C11" s="114"/>
+      <c r="D11" s="114"/>
+      <c r="E11" s="114"/>
+      <c r="F11" s="114"/>
+      <c r="G11" s="114"/>
+      <c r="H11" s="114"/>
+      <c r="I11" s="114"/>
+      <c r="J11" s="114"/>
+      <c r="K11" s="114"/>
+      <c r="L11" s="114"/>
     </row>
     <row r="12" spans="1:12" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="28"/>
-      <c r="B12" s="107">
+      <c r="B12" s="115">
         <v>0</v>
       </c>
-      <c r="C12" s="107"/>
+      <c r="C12" s="115"/>
       <c r="D12" s="57"/>
       <c r="E12" s="65"/>
       <c r="F12" s="57"/>
-      <c r="G12" s="108" t="s">
+      <c r="G12" s="116" t="s">
         <v>187</v>
       </c>
-      <c r="H12" s="108"/>
-      <c r="I12" s="108"/>
-      <c r="J12" s="108"/>
-      <c r="K12" s="108"/>
-      <c r="L12" s="108"/>
+      <c r="H12" s="116"/>
+      <c r="I12" s="116"/>
+      <c r="J12" s="116"/>
+      <c r="K12" s="116"/>
+      <c r="L12" s="116"/>
     </row>
     <row r="13" spans="1:12" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="26"/>
-      <c r="B13" s="107">
+      <c r="B13" s="115">
         <v>0</v>
       </c>
-      <c r="C13" s="107"/>
-      <c r="G13" s="108" t="s">
+      <c r="C13" s="115"/>
+      <c r="G13" s="116" t="s">
         <v>188</v>
       </c>
-      <c r="H13" s="108"/>
-      <c r="I13" s="108"/>
-      <c r="J13" s="108"/>
-      <c r="K13" s="108"/>
-      <c r="L13" s="108"/>
+      <c r="H13" s="116"/>
+      <c r="I13" s="116"/>
+      <c r="J13" s="116"/>
+      <c r="K13" s="116"/>
+      <c r="L13" s="116"/>
     </row>
     <row r="14" spans="1:12" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="72"/>
-      <c r="H14" s="104" t="s">
+      <c r="H14" s="112" t="s">
         <v>189</v>
       </c>
-      <c r="I14" s="104"/>
-      <c r="J14" s="104"/>
-      <c r="K14" s="104"/>
-      <c r="L14" s="104"/>
+      <c r="I14" s="112"/>
+      <c r="J14" s="112"/>
+      <c r="K14" s="112"/>
+      <c r="L14" s="112"/>
     </row>
     <row r="15" spans="1:12" s="72" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="28"/>
-      <c r="B15" s="105" t="s">
+      <c r="B15" s="113" t="s">
         <v>190</v>
       </c>
-      <c r="C15" s="105"/>
-      <c r="D15" s="105"/>
-      <c r="E15" s="105"/>
+      <c r="C15" s="113"/>
+      <c r="D15" s="113"/>
+      <c r="E15" s="113"/>
       <c r="I15"/>
     </row>
     <row r="16" spans="1:12" s="72" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="28"/>
-      <c r="B16" s="104" t="s">
+      <c r="B16" s="112" t="s">
         <v>191</v>
       </c>
-      <c r="C16" s="104"/>
-      <c r="D16" s="104"/>
-      <c r="E16" s="104"/>
+      <c r="C16" s="112"/>
+      <c r="D16" s="112"/>
+      <c r="E16" s="112"/>
       <c r="F16" s="69"/>
       <c r="G16" s="69"/>
       <c r="H16" s="69"/>
@@ -5182,12 +5182,14 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A6:L6"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="B16:E16"/>
+    <mergeCell ref="A11:L11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="G12:L12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="G13:L13"/>
+    <mergeCell ref="H14:L14"/>
     <mergeCell ref="A7:L7"/>
     <mergeCell ref="A8:A9"/>
     <mergeCell ref="B8:B9"/>
@@ -5198,14 +5200,12 @@
     <mergeCell ref="G8:J8"/>
     <mergeCell ref="K8:K9"/>
     <mergeCell ref="L8:L9"/>
-    <mergeCell ref="B15:E15"/>
-    <mergeCell ref="B16:E16"/>
-    <mergeCell ref="A11:L11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="G12:L12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="G13:L13"/>
-    <mergeCell ref="H14:L14"/>
+    <mergeCell ref="A6:L6"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5236,156 +5236,156 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="113" t="s">
+      <c r="A1" s="103" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="113"/>
-      <c r="C1" s="113"/>
-      <c r="D1" s="113"/>
-      <c r="E1" s="113"/>
-      <c r="F1" s="113"/>
-      <c r="G1" s="113"/>
-      <c r="H1" s="113"/>
-      <c r="I1" s="113"/>
-      <c r="J1" s="113"/>
-      <c r="K1" s="113"/>
-      <c r="L1" s="113"/>
+      <c r="B1" s="103"/>
+      <c r="C1" s="103"/>
+      <c r="D1" s="103"/>
+      <c r="E1" s="103"/>
+      <c r="F1" s="103"/>
+      <c r="G1" s="103"/>
+      <c r="H1" s="103"/>
+      <c r="I1" s="103"/>
+      <c r="J1" s="103"/>
+      <c r="K1" s="103"/>
+      <c r="L1" s="103"/>
     </row>
     <row r="2" spans="1:12" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="114" t="s">
+      <c r="A2" s="104" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="115"/>
-      <c r="C2" s="115"/>
-      <c r="D2" s="115"/>
-      <c r="E2" s="115"/>
-      <c r="F2" s="115"/>
-      <c r="G2" s="115"/>
-      <c r="H2" s="115"/>
-      <c r="I2" s="115"/>
-      <c r="J2" s="115"/>
-      <c r="K2" s="115"/>
-      <c r="L2" s="115"/>
+      <c r="B2" s="105"/>
+      <c r="C2" s="105"/>
+      <c r="D2" s="105"/>
+      <c r="E2" s="105"/>
+      <c r="F2" s="105"/>
+      <c r="G2" s="105"/>
+      <c r="H2" s="105"/>
+      <c r="I2" s="105"/>
+      <c r="J2" s="105"/>
+      <c r="K2" s="105"/>
+      <c r="L2" s="105"/>
     </row>
     <row r="3" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="116">
+      <c r="A3" s="106">
         <v>3</v>
       </c>
-      <c r="B3" s="116"/>
-      <c r="C3" s="116"/>
-      <c r="D3" s="116"/>
-      <c r="E3" s="116"/>
-      <c r="F3" s="116"/>
-      <c r="G3" s="116"/>
-      <c r="H3" s="116"/>
-      <c r="I3" s="116"/>
-      <c r="J3" s="116"/>
-      <c r="K3" s="116"/>
-      <c r="L3" s="116"/>
+      <c r="B3" s="106"/>
+      <c r="C3" s="106"/>
+      <c r="D3" s="106"/>
+      <c r="E3" s="106"/>
+      <c r="F3" s="106"/>
+      <c r="G3" s="106"/>
+      <c r="H3" s="106"/>
+      <c r="I3" s="106"/>
+      <c r="J3" s="106"/>
+      <c r="K3" s="106"/>
+      <c r="L3" s="106"/>
     </row>
     <row r="4" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="117" t="s">
+      <c r="A4" s="107" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="117"/>
-      <c r="C4" s="117"/>
-      <c r="D4" s="117"/>
-      <c r="E4" s="117"/>
-      <c r="F4" s="117"/>
-      <c r="G4" s="117"/>
-      <c r="H4" s="117"/>
-      <c r="I4" s="117"/>
-      <c r="J4" s="117"/>
-      <c r="K4" s="117"/>
+      <c r="B4" s="107"/>
+      <c r="C4" s="107"/>
+      <c r="D4" s="107"/>
+      <c r="E4" s="107"/>
+      <c r="F4" s="107"/>
+      <c r="G4" s="107"/>
+      <c r="H4" s="107"/>
+      <c r="I4" s="107"/>
+      <c r="J4" s="107"/>
+      <c r="K4" s="107"/>
       <c r="L4" s="6"/>
     </row>
     <row r="5" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="117" t="s">
+      <c r="A5" s="107" t="s">
         <v>41</v>
       </c>
-      <c r="B5" s="117"/>
-      <c r="C5" s="117"/>
-      <c r="D5" s="117"/>
-      <c r="E5" s="117"/>
-      <c r="F5" s="117"/>
-      <c r="G5" s="117"/>
-      <c r="H5" s="117"/>
-      <c r="I5" s="117"/>
-      <c r="J5" s="117"/>
-      <c r="K5" s="117"/>
+      <c r="B5" s="107"/>
+      <c r="C5" s="107"/>
+      <c r="D5" s="107"/>
+      <c r="E5" s="107"/>
+      <c r="F5" s="107"/>
+      <c r="G5" s="107"/>
+      <c r="H5" s="107"/>
+      <c r="I5" s="107"/>
+      <c r="J5" s="107"/>
+      <c r="K5" s="107"/>
       <c r="L5" s="6"/>
     </row>
     <row r="6" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="109" t="s">
+      <c r="A6" s="108" t="s">
         <v>193</v>
       </c>
-      <c r="B6" s="109"/>
-      <c r="C6" s="109"/>
-      <c r="D6" s="109"/>
-      <c r="E6" s="109"/>
-      <c r="F6" s="109"/>
-      <c r="G6" s="109"/>
-      <c r="H6" s="109"/>
-      <c r="I6" s="109"/>
-      <c r="J6" s="109"/>
-      <c r="K6" s="109"/>
-      <c r="L6" s="109"/>
+      <c r="B6" s="108"/>
+      <c r="C6" s="108"/>
+      <c r="D6" s="108"/>
+      <c r="E6" s="108"/>
+      <c r="F6" s="108"/>
+      <c r="G6" s="108"/>
+      <c r="H6" s="108"/>
+      <c r="I6" s="108"/>
+      <c r="J6" s="108"/>
+      <c r="K6" s="108"/>
+      <c r="L6" s="108"/>
     </row>
     <row r="7" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="109" t="s">
+      <c r="A7" s="108" t="s">
         <v>176</v>
       </c>
-      <c r="B7" s="109"/>
-      <c r="C7" s="109"/>
-      <c r="D7" s="109"/>
-      <c r="E7" s="109"/>
-      <c r="F7" s="109"/>
-      <c r="G7" s="109"/>
-      <c r="H7" s="109"/>
-      <c r="I7" s="109"/>
-      <c r="J7" s="109"/>
-      <c r="K7" s="109"/>
-      <c r="L7" s="109"/>
+      <c r="B7" s="108"/>
+      <c r="C7" s="108"/>
+      <c r="D7" s="108"/>
+      <c r="E7" s="108"/>
+      <c r="F7" s="108"/>
+      <c r="G7" s="108"/>
+      <c r="H7" s="108"/>
+      <c r="I7" s="108"/>
+      <c r="J7" s="108"/>
+      <c r="K7" s="108"/>
+      <c r="L7" s="108"/>
     </row>
     <row r="8" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="110" t="s">
+      <c r="A8" s="109" t="s">
         <v>177</v>
       </c>
-      <c r="B8" s="110" t="s">
+      <c r="B8" s="109" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="110" t="s">
+      <c r="C8" s="109" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="110" t="s">
+      <c r="D8" s="109" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="111" t="s">
+      <c r="E8" s="110" t="s">
         <v>11</v>
       </c>
-      <c r="F8" s="110" t="s">
+      <c r="F8" s="109" t="s">
         <v>178</v>
       </c>
-      <c r="G8" s="112" t="s">
+      <c r="G8" s="111" t="s">
         <v>179</v>
       </c>
-      <c r="H8" s="110"/>
-      <c r="I8" s="110"/>
-      <c r="J8" s="110"/>
-      <c r="K8" s="110" t="s">
+      <c r="H8" s="109"/>
+      <c r="I8" s="109"/>
+      <c r="J8" s="109"/>
+      <c r="K8" s="109" t="s">
         <v>12</v>
       </c>
-      <c r="L8" s="110" t="s">
+      <c r="L8" s="109" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="25.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="110"/>
-      <c r="B9" s="110"/>
-      <c r="C9" s="110"/>
-      <c r="D9" s="110"/>
-      <c r="E9" s="111"/>
-      <c r="F9" s="110"/>
+      <c r="A9" s="109"/>
+      <c r="B9" s="109"/>
+      <c r="C9" s="109"/>
+      <c r="D9" s="109"/>
+      <c r="E9" s="110"/>
+      <c r="F9" s="109"/>
       <c r="G9" s="70" t="s">
         <v>180</v>
       </c>
@@ -5398,10 +5398,10 @@
       <c r="J9" s="71" t="s">
         <v>182</v>
       </c>
-      <c r="K9" s="110"/>
-      <c r="L9" s="110"/>
-    </row>
-    <row r="10" spans="1:12" ht="16.899999999999999" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K9" s="109"/>
+      <c r="L9" s="109"/>
+    </row>
+    <row r="10" spans="1:12" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="62">
         <v>1</v>
       </c>
@@ -5419,7 +5419,7 @@
       </c>
       <c r="F10" s="67">
         <f ca="1">IF(E10 &lt;&gt; "",YEAR(NOW())-YEAR(E10), "")</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G10" s="90" t="s">
         <v>185</v>
@@ -5432,83 +5432,83 @@
       <c r="K10" s="63" t="s">
         <v>186</v>
       </c>
-      <c r="L10" s="93"/>
+      <c r="L10" s="63"/>
     </row>
     <row r="11" spans="1:12" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="106"/>
-      <c r="B11" s="106"/>
-      <c r="C11" s="106"/>
-      <c r="D11" s="106"/>
-      <c r="E11" s="106"/>
-      <c r="F11" s="106"/>
-      <c r="G11" s="106"/>
-      <c r="H11" s="106"/>
-      <c r="I11" s="106"/>
-      <c r="J11" s="106"/>
-      <c r="K11" s="106"/>
-      <c r="L11" s="106"/>
+      <c r="A11" s="114"/>
+      <c r="B11" s="114"/>
+      <c r="C11" s="114"/>
+      <c r="D11" s="114"/>
+      <c r="E11" s="114"/>
+      <c r="F11" s="114"/>
+      <c r="G11" s="114"/>
+      <c r="H11" s="114"/>
+      <c r="I11" s="114"/>
+      <c r="J11" s="114"/>
+      <c r="K11" s="114"/>
+      <c r="L11" s="114"/>
     </row>
     <row r="12" spans="1:12" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="28"/>
-      <c r="B12" s="107">
+      <c r="B12" s="115">
         <v>0</v>
       </c>
-      <c r="C12" s="107"/>
+      <c r="C12" s="115"/>
       <c r="D12" s="57"/>
       <c r="E12" s="65"/>
       <c r="F12" s="57"/>
-      <c r="G12" s="108" t="s">
+      <c r="G12" s="116" t="s">
         <v>187</v>
       </c>
-      <c r="H12" s="108"/>
-      <c r="I12" s="108"/>
-      <c r="J12" s="108"/>
-      <c r="K12" s="108"/>
-      <c r="L12" s="108"/>
+      <c r="H12" s="116"/>
+      <c r="I12" s="116"/>
+      <c r="J12" s="116"/>
+      <c r="K12" s="116"/>
+      <c r="L12" s="116"/>
     </row>
     <row r="13" spans="1:12" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="26"/>
-      <c r="B13" s="107">
+      <c r="B13" s="115">
         <v>0</v>
       </c>
-      <c r="C13" s="107"/>
-      <c r="G13" s="108" t="s">
+      <c r="C13" s="115"/>
+      <c r="G13" s="116" t="s">
         <v>188</v>
       </c>
-      <c r="H13" s="108"/>
-      <c r="I13" s="108"/>
-      <c r="J13" s="108"/>
-      <c r="K13" s="108"/>
-      <c r="L13" s="108"/>
+      <c r="H13" s="116"/>
+      <c r="I13" s="116"/>
+      <c r="J13" s="116"/>
+      <c r="K13" s="116"/>
+      <c r="L13" s="116"/>
     </row>
     <row r="14" spans="1:12" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="72"/>
-      <c r="H14" s="104" t="s">
+      <c r="H14" s="112" t="s">
         <v>189</v>
       </c>
-      <c r="I14" s="104"/>
-      <c r="J14" s="104"/>
-      <c r="K14" s="104"/>
-      <c r="L14" s="104"/>
+      <c r="I14" s="112"/>
+      <c r="J14" s="112"/>
+      <c r="K14" s="112"/>
+      <c r="L14" s="112"/>
     </row>
     <row r="15" spans="1:12" s="72" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="28"/>
-      <c r="B15" s="105" t="s">
+      <c r="B15" s="113" t="s">
         <v>190</v>
       </c>
-      <c r="C15" s="105"/>
-      <c r="D15" s="105"/>
-      <c r="E15" s="105"/>
+      <c r="C15" s="113"/>
+      <c r="D15" s="113"/>
+      <c r="E15" s="113"/>
       <c r="I15"/>
     </row>
     <row r="16" spans="1:12" s="72" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="28"/>
-      <c r="B16" s="104" t="s">
+      <c r="B16" s="112" t="s">
         <v>191</v>
       </c>
-      <c r="C16" s="104"/>
-      <c r="D16" s="104"/>
-      <c r="E16" s="104"/>
+      <c r="C16" s="112"/>
+      <c r="D16" s="112"/>
+      <c r="E16" s="112"/>
       <c r="F16" s="69"/>
       <c r="G16" s="69"/>
       <c r="H16" s="69"/>
@@ -5835,12 +5835,14 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A6:L6"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="B16:E16"/>
+    <mergeCell ref="A11:L11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="G12:L12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="G13:L13"/>
+    <mergeCell ref="H14:L14"/>
     <mergeCell ref="A7:L7"/>
     <mergeCell ref="A8:A9"/>
     <mergeCell ref="B8:B9"/>
@@ -5851,14 +5853,12 @@
     <mergeCell ref="G8:J8"/>
     <mergeCell ref="K8:K9"/>
     <mergeCell ref="L8:L9"/>
-    <mergeCell ref="B15:E15"/>
-    <mergeCell ref="B16:E16"/>
-    <mergeCell ref="A11:L11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="G12:L12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="G13:L13"/>
-    <mergeCell ref="H14:L14"/>
+    <mergeCell ref="A6:L6"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5890,98 +5890,98 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A1" s="101" t="s">
+      <c r="A1" s="100" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="101"/>
-      <c r="C1" s="101"/>
-      <c r="D1" s="101"/>
-      <c r="E1" s="101"/>
-      <c r="F1" s="101"/>
-      <c r="G1" s="101"/>
-      <c r="H1" s="101"/>
-      <c r="I1" s="101"/>
-      <c r="J1" s="101"/>
-      <c r="K1" s="101"/>
-      <c r="L1" s="101"/>
-      <c r="M1" s="101"/>
+      <c r="B1" s="100"/>
+      <c r="C1" s="100"/>
+      <c r="D1" s="100"/>
+      <c r="E1" s="100"/>
+      <c r="F1" s="100"/>
+      <c r="G1" s="100"/>
+      <c r="H1" s="100"/>
+      <c r="I1" s="100"/>
+      <c r="J1" s="100"/>
+      <c r="K1" s="100"/>
+      <c r="L1" s="100"/>
+      <c r="M1" s="100"/>
     </row>
     <row r="2" spans="1:14" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="95" t="s">
+      <c r="A2" s="94" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="118"/>
-      <c r="C2" s="118"/>
-      <c r="D2" s="118"/>
-      <c r="E2" s="118"/>
-      <c r="F2" s="118"/>
-      <c r="G2" s="118"/>
-      <c r="H2" s="118"/>
-      <c r="I2" s="118"/>
-      <c r="J2" s="118"/>
-      <c r="K2" s="118"/>
-      <c r="L2" s="118"/>
-      <c r="M2" s="118"/>
+      <c r="B2" s="117"/>
+      <c r="C2" s="117"/>
+      <c r="D2" s="117"/>
+      <c r="E2" s="117"/>
+      <c r="F2" s="117"/>
+      <c r="G2" s="117"/>
+      <c r="H2" s="117"/>
+      <c r="I2" s="117"/>
+      <c r="J2" s="117"/>
+      <c r="K2" s="117"/>
+      <c r="L2" s="117"/>
+      <c r="M2" s="117"/>
     </row>
     <row r="3" spans="1:14" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="116">
+      <c r="A3" s="106">
         <v>3</v>
       </c>
-      <c r="B3" s="116"/>
-      <c r="C3" s="116"/>
-      <c r="D3" s="116"/>
-      <c r="E3" s="116"/>
-      <c r="F3" s="116"/>
-      <c r="G3" s="116"/>
-      <c r="H3" s="116"/>
-      <c r="I3" s="116"/>
-      <c r="J3" s="116"/>
-      <c r="K3" s="116"/>
-      <c r="L3" s="116"/>
-      <c r="M3" s="116"/>
+      <c r="B3" s="106"/>
+      <c r="C3" s="106"/>
+      <c r="D3" s="106"/>
+      <c r="E3" s="106"/>
+      <c r="F3" s="106"/>
+      <c r="G3" s="106"/>
+      <c r="H3" s="106"/>
+      <c r="I3" s="106"/>
+      <c r="J3" s="106"/>
+      <c r="K3" s="106"/>
+      <c r="L3" s="106"/>
+      <c r="M3" s="106"/>
     </row>
     <row r="5" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A5" s="103" t="s">
+      <c r="A5" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="103"/>
-      <c r="C5" s="103"/>
-      <c r="D5" s="103"/>
-      <c r="E5" s="103"/>
-      <c r="F5" s="103"/>
+      <c r="B5" s="102"/>
+      <c r="C5" s="102"/>
+      <c r="D5" s="102"/>
+      <c r="E5" s="102"/>
+      <c r="F5" s="102"/>
       <c r="G5" s="31"/>
     </row>
     <row r="6" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A6" s="103" t="s">
+      <c r="A6" s="102" t="s">
         <v>41</v>
       </c>
-      <c r="B6" s="103"/>
-      <c r="C6" s="103"/>
-      <c r="D6" s="103"/>
-      <c r="E6" s="103"/>
-      <c r="F6" s="103"/>
+      <c r="B6" s="102"/>
+      <c r="C6" s="102"/>
+      <c r="D6" s="102"/>
+      <c r="E6" s="102"/>
+      <c r="F6" s="102"/>
       <c r="G6" s="31"/>
     </row>
     <row r="7" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.65">
       <c r="D7" s="1"/>
-      <c r="E7" s="101" t="s">
+      <c r="E7" s="100" t="s">
         <v>194</v>
       </c>
-      <c r="F7" s="101"/>
-      <c r="G7" s="101"/>
-      <c r="H7" s="101"/>
-      <c r="I7" s="101"/>
+      <c r="F7" s="100"/>
+      <c r="G7" s="100"/>
+      <c r="H7" s="100"/>
+      <c r="I7" s="100"/>
       <c r="J7" s="2"/>
     </row>
     <row r="8" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.65">
       <c r="D8" s="1"/>
-      <c r="E8" s="101" t="s">
+      <c r="E8" s="100" t="s">
         <v>6</v>
       </c>
-      <c r="F8" s="101"/>
-      <c r="G8" s="101"/>
-      <c r="H8" s="101"/>
-      <c r="I8" s="101"/>
+      <c r="F8" s="100"/>
+      <c r="G8" s="100"/>
+      <c r="H8" s="100"/>
+      <c r="I8" s="100"/>
       <c r="J8" s="2"/>
     </row>
     <row r="9" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>